<commit_message>
Rework partners account per owner's classification
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WA2XXv3viuKc4AVC546mfn
</commit_message>
<xml_diff>
--- a/حساب_الشريكين_مع_مزرعة_الرياض.xlsx
+++ b/حساب_الشريكين_مع_مزرعة_الرياض.xlsx
@@ -10,7 +10,7 @@
     <sheet name="ملخص الشركاء" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="أبو خالد - بساتين الرياض" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="أبو مازن - نسما الشرق (تبوك)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="بنود تحتاج تحديد الممول" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="إيرادات ومصروفات قبل الفترة" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="تحقق مسحوبات أبو خالد 24.2-3.6" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
@@ -104,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -148,6 +148,12 @@
     <xf numFmtId="4" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -514,13 +520,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="54" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="56" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -533,27 +539,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>أبو خالد = مؤسسة بساتين الرياض | أبو مازن = شركة نسما الشرق (مزرعة تبوك) – الشريكان في مزرعة الرياض</t>
+          <t>أبو خالد = مؤسسة بساتين الرياض | أبو مازن = شركة نسما الشرق (مزرعة تبوك)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="24" t="inlineStr">
         <is>
           <t>البند</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>أبو خالد – بساتين الرياض</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="24" t="inlineStr">
         <is>
           <t>أبو مازن – نسما الشرق</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="24" t="inlineStr">
         <is>
           <t>ملاحظة</t>
         </is>
@@ -562,7 +568,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>1) المسحوبات المباشرة من المزرعة (مديونية عليه)</t>
+          <t>1) المسحوبات المباشرة</t>
         </is>
       </c>
       <c r="B5" s="4">
@@ -573,24 +579,20 @@
         <f>'أبو مازن - نسما الشرق (تبوك)'!C9</f>
         <v/>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>بضاعة مسحوبة/مباعة لحسابه</t>
-        </is>
-      </c>
+      <c r="D5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2) المسحوبات النقدية من خزنة المزرعة (مديونية عليه)</t>
+          <t>2) المسحوبات النقدية</t>
         </is>
       </c>
       <c r="B6" s="4">
-        <f>'أبو خالد - بساتين الرياض'!C21</f>
+        <f>'أبو خالد - بساتين الرياض'!C12</f>
         <v/>
       </c>
       <c r="C6" s="4">
-        <f>'أبو مازن - نسما الشرق (تبوك)'!C24</f>
+        <f>'أبو مازن - نسما الشرق (تبوك)'!C16</f>
         <v/>
       </c>
       <c r="D6" s="3" t="inlineStr"/>
@@ -598,7 +600,7 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>إجمالي المديونية عليه</t>
+          <t>إجمالي المسحوبات (عليه)</t>
         </is>
       </c>
       <c r="B7" s="6">
@@ -614,116 +616,78 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>3) الدعم المقدم للمزرعة (حق له)</t>
+          <t>3) سدادات لمسحوباته مسجلة بكشف الخزنة</t>
         </is>
       </c>
       <c r="B8" s="4">
-        <f>'أبو خالد - بساتين الرياض'!C15</f>
-        <v/>
-      </c>
-      <c r="C8" s="4">
-        <f>'أبو مازن - نسما الشرق (تبوك)'!C19</f>
-        <v/>
+        <f>'أبو خالد - بساتين الرياض'!C17</f>
+        <v/>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>مصروفات وسدادات ومشتريات دفعها عن المزرعة</t>
+          <t>توريدات وسدادات أبو خالد</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>الصافي المبدئي (موجب = مديونية عليه للمزرعة / سالب = مستحق له)</t>
-        </is>
-      </c>
-      <c r="B9" s="6">
-        <f>B7-B8</f>
-        <v/>
-      </c>
-      <c r="C9" s="6">
-        <f>C7-C8</f>
-        <v/>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>⚠ مبدئي – قبل تحديد ممول بنود التأسيس والتشغيل قبل الفترة (1,368,006.47) وأسعار مسحوبات قبل الفترة</t>
-        </is>
-      </c>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>4) الدعم المقدم للمزرعة</t>
+        </is>
+      </c>
+      <c r="B9" s="4">
+        <f>'أبو خالد - بساتين الرياض'!C24</f>
+        <v/>
+      </c>
+      <c r="C9" s="4">
+        <f>'أبو مازن - نسما الشرق (تبوك)'!C26</f>
+        <v/>
+      </c>
+      <c r="D9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>إجمالي ما له (سدادات + دعم)</t>
+        </is>
+      </c>
+      <c r="B10" s="6">
+        <f>B8+B9</f>
+        <v/>
+      </c>
+      <c r="C10" s="6">
+        <f>C8+C9</f>
+        <v/>
+      </c>
+      <c r="D10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>بنود لم تُوزع بعد على الشريكين</t>
-        </is>
-      </c>
-      <c r="B11" s="8">
-        <f>'بنود تحتاج تحديد الممول'!C7</f>
-        <v/>
-      </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>مصروفات التأسيس من البنوك + تشغيل قبل الفترة – يلزم تحديد من دفعها</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="9" t="inlineStr"/>
-    </row>
-    <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>ملاحظات أساسية:</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>1) حساب أبو خالد: كشف الخزنة يُظهر لحسابه مبيعات 600,335.25 وسدادات 763,323.81 (رصيد دائن 162,988.56 لصالحه) – الفرق عن 761,583.25 هنا لأن الكشف سجّل عقد عرعر بالمسلّم 367,803.75 وسجّل ما قبل 1-11-2025 كقيد تسوية 62,937.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>2) سند مسحوبات بساتين الرياض (24.2–3.6.2026) كله من عقود أبو خالد ومدرج في مبيعاته – لا يُضاف مرة أخرى. التفاصيل في شيت التحقق.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="40" customHeight="1">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>3) مسحوبات نسما من الرياض محسوبة بقيم النظام (426,293.23). لو اعتُمدت أسعار التحويل الخاصة بالمحاسب فالرقم يتغير – يلزم الاتفاق على الأسعار.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="40" customHeight="1">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>4) مبلغ 100,000 المنصرف لأبو خالد كان "بتعليمات أبو مازن".</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="40" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
-        <is>
-          <t>5) لم تُحتسب هنا: أرصدة عهد لم تُسوَّ (1,543.91)، ومديونيات الموردين الخارجيين (الجزيرة 21,250) لأنها ليست على أي من الشريكين.</t>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>الصافي (موجب = مديونية عليه للمزرعة / سالب = مستحق له)</t>
+        </is>
+      </c>
+      <c r="B11" s="6">
+        <f>B7-B10</f>
+        <v/>
+      </c>
+      <c r="C11" s="6">
+        <f>C7-C10</f>
+        <v/>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>⚠ لم تُسعّر بعد مسحوبات تبوك قبل الفترة (102,875 حبة)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A15:D15"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A16:D16"/>
-    <mergeCell ref="A13:D13"/>
-    <mergeCell ref="A14:D14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -735,13 +699,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
     <col width="70" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -755,32 +719,32 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>أولاً: المسحوبات المباشرة من مزرعة الرياض (مديونية على أبو خالد)</t>
+          <t>أولاً: المسحوبات المباشرة (مديونية على أبو خالد)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="25" t="inlineStr">
         <is>
           <t>م</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="25" t="inlineStr">
         <is>
           <t>البند</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="25" t="inlineStr">
         <is>
           <t>المبلغ</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="D4" s="25" t="inlineStr">
         <is>
           <t>المصدر</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
+      <c r="E4" s="25" t="inlineStr">
         <is>
           <t>ملاحظة</t>
         </is>
@@ -792,43 +756,39 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>مبيعات/مسحوبات عقود WHK (30-7-2025 إلى 31-7-2026) شاملة عقد عرعر بالقيمة الكاملة 440,000</t>
+          <t>عقد عرعر WHK-2364 بالقيمة الكاملة</t>
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>761583.25</v>
+        <v>440000</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>ملف إجمالي مبيعات المناديب – مبيعات أبو خالد</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>47 عقد – منها بنود سند المسحوبات 24.2–3.6.2026 (مدرجة ضمنها ولا تُحسب مرتين)</t>
-        </is>
-      </c>
+          <t>ملف المبيعات – مبيعات أبو خالد</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="n">
+      <c r="A6" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>مبيعات مزرعة الرياض قبل الفترة (1-10-2024 إلى 30-6-2025)</t>
-        </is>
-      </c>
-      <c r="C6" s="13" t="n">
-        <v>610688</v>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>ملف المبيعات – شيت مبيعات قبل 30.7.2025</t>
-        </is>
-      </c>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>⚠ مفترض أن أبو خالد هو من حصّل هذه المبيعات (لأن مصروفات الفترة دُفعت منه "من المبيعات") – يلزم التأكيد</t>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>مبيعات المندوب أبو خالد – باقي عقود WHK (46 عقد) من 30-7-2025 إلى 31-7-2026</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>321583.25</v>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>ملف المبيعات – مبيعات أبو خالد</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>تشمل بنود سند المسحوبات 24.2–3.6.2026 (لا تُحسب مرتين)</t>
         </is>
       </c>
     </row>
@@ -849,234 +809,269 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>ثانياً: المبالغ التي دعم بها أبو خالد مزرعة الرياض (حق لأبو خالد)</t>
+          <t>ثانياً: المسحوبات النقدية من خزنة المزرعة (مديونية على أبو خالد)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="25" t="inlineStr">
         <is>
           <t>م</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="25" t="inlineStr">
         <is>
           <t>البند</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="25" t="inlineStr">
         <is>
           <t>المبلغ</t>
         </is>
       </c>
-      <c r="D10" s="11" t="inlineStr">
+      <c r="D10" s="25" t="inlineStr">
         <is>
           <t>المصدر</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr">
+      <c r="E10" s="25" t="inlineStr">
         <is>
           <t>ملاحظة</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n">
+      <c r="A11" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>مصروفات تشغيل دفعها من المبيعات (10-2024 إلى 6-2025)</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>413236</v>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>ملف المصاريف التشغيلية – مصروفات قبل 30.7.2025</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>إجماليات ربع سنوية بدون تفصيل</t>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>تسديد لأبو خالد من المديونية (18-5-2026)</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>كشف الخزنة – مستند 156</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>⚠ مسجل على حساب أبو خالد – يلزم التأكيد إن كان يخصه أو يخص أبو مازن</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="n">
+      <c r="A12" s="14" t="inlineStr"/>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>الإجمالي</t>
+        </is>
+      </c>
+      <c r="C12" s="15">
+        <f>SUM(C11:C11)</f>
+        <v/>
+      </c>
+      <c r="D12" s="14" t="n"/>
+      <c r="E12" s="14" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>ثالثاً: سدادات أبو خالد لمسحوباته (مسجلة لحسابه في كشف الخزنة)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="25" t="inlineStr">
+        <is>
+          <t>م</t>
+        </is>
+      </c>
+      <c r="B15" s="25" t="inlineStr">
+        <is>
+          <t>البند</t>
+        </is>
+      </c>
+      <c r="C15" s="25" t="inlineStr">
+        <is>
+          <t>المبلغ</t>
+        </is>
+      </c>
+      <c r="D15" s="25" t="inlineStr">
+        <is>
+          <t>المصدر</t>
+        </is>
+      </c>
+      <c r="E15" s="25" t="inlineStr">
+        <is>
+          <t>ملاحظة</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>توريدات نقدية وسدادات مسجلة لحسابه (Cash Payment)</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>763323.8100000001</v>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>كشف الحساب – عميل 5000</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>سداد لمسحوباته وليست دعماً. تشمل توريدات نقدية من المبيعات + مشتريات دفعها عن المزرعة (زهور الجزيرة لعقد عرعر 199,353 – بذور بساتين قديم 147,745.75 – بيتموس 53,475 – جهنمية وسايكس 49,550 – غرس نجد 14,515 – مراكن 20,000 ...)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr"/>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>الإجمالي</t>
+        </is>
+      </c>
+      <c r="C17" s="15">
+        <f>SUM(C16:C16)</f>
+        <v/>
+      </c>
+      <c r="D17" s="14" t="n"/>
+      <c r="E17" s="14" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>رابعاً: دعم أبو خالد لمزرعة الرياض (حق له)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="25" t="inlineStr">
+        <is>
+          <t>م</t>
+        </is>
+      </c>
+      <c r="B20" s="25" t="inlineStr">
+        <is>
+          <t>البند</t>
+        </is>
+      </c>
+      <c r="C20" s="25" t="inlineStr">
+        <is>
+          <t>المبلغ</t>
+        </is>
+      </c>
+      <c r="D20" s="25" t="inlineStr">
+        <is>
+          <t>المصدر</t>
+        </is>
+      </c>
+      <c r="E20" s="25" t="inlineStr">
+        <is>
+          <t>ملاحظة</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>ضخ نقدي في مصاريف تشغيل المزرعة</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>189235</v>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>بيان صاحب الحساب</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>سدادات وتوريدات نقدية مسجلة لحسابه بكشف الخزنة (Cash Payment)</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="n">
-        <v>763323.8100000001</v>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>كشف الحساب – عميل 5000</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>تشمل: توريدات نقدية من المبيعات + سداد مشتريات عن المزرعة (زهور الجزيرة 196,225 – بذور بساتين قديم 147,745.75 – جهنمية 37,550 – سايكس 12,000 – غرس نجد 14,515 – بيتموس 53,475 – مراكن 20,000 ...)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="n">
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>أوامر شراء بساتين الرياض غير مسددة – PO-1023</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>33950</v>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>ملف أوامر الشراء 2026</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>أوامر شراء من بساتين الرياض لم تُسدد – PO-1023</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="n">
-        <v>33950</v>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>أوامر شراء بساتين الرياض مدفوعة جزئياً – PO-0777</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="n">
+        <v>66420</v>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
         <is>
           <t>ملف أوامر الشراء 2026</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>غير مدفوع – مستلم بالكامل</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="B14" s="12" t="inlineStr">
-        <is>
-          <t>أوامر شراء من بساتين الرياض مدفوعة جزئياً – PO-0777</t>
-        </is>
-      </c>
-      <c r="C14" s="13" t="n">
-        <v>66420</v>
-      </c>
-      <c r="D14" s="12" t="inlineStr">
-        <is>
-          <t>ملف أوامر الشراء 2026</t>
-        </is>
-      </c>
-      <c r="E14" s="12" t="inlineStr">
-        <is>
-          <t>⚠ القيمة كاملة – يُخصم منها المسدد عند معرفته</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="14" t="inlineStr"/>
-      <c r="B15" s="14" t="inlineStr">
+      <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>⚠ القيمة كاملة – يُخصم المسدد عند معرفته</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr"/>
+      <c r="B24" s="14" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="C15" s="15">
-        <f>SUM(C11:C14)</f>
-        <v/>
-      </c>
-      <c r="D15" s="14" t="n"/>
-      <c r="E15" s="14" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>ثالثاً: مسحوبات نقدية من خزنة مزرعة الرياض (مديونية على أبو خالد)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="11" t="inlineStr">
-        <is>
-          <t>م</t>
-        </is>
-      </c>
-      <c r="B18" s="11" t="inlineStr">
-        <is>
-          <t>البند</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="inlineStr">
-        <is>
-          <t>المبلغ</t>
-        </is>
-      </c>
-      <c r="D18" s="11" t="inlineStr">
-        <is>
-          <t>المصدر</t>
-        </is>
-      </c>
-      <c r="E18" s="11" t="inlineStr">
-        <is>
-          <t>ملاحظة</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>منصرف لأبو خالد بتعليمات أبو مازن (9-3-2026)</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="n">
-        <v>100000</v>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>كشف الخزنة – مصروف رقم 131</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>تسديد لأبو خالد من المديونية (18-5-2026)</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="n">
-        <v>2000</v>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>كشف الخزنة – مستند 156 على حسابه</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="14" t="inlineStr"/>
-      <c r="B21" s="14" t="inlineStr">
-        <is>
-          <t>الإجمالي</t>
-        </is>
-      </c>
-      <c r="C21" s="15">
-        <f>SUM(C19:C20)</f>
-        <v/>
-      </c>
-      <c r="D21" s="14" t="n"/>
-      <c r="E21" s="14" t="n"/>
+      <c r="C24" s="15">
+        <f>SUM(C21:C23)</f>
+        <v/>
+      </c>
+      <c r="D24" s="14" t="n"/>
+      <c r="E24" s="14" t="n"/>
+    </row>
+    <row r="26" ht="32" customHeight="1">
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" s="23" t="inlineStr">
+        <is>
+          <t>ملاحظة: أوامر بساتين المسددة (PO-288 و PO-287-REV1 = 147,745.75 سُددت كتسوية على حسابه، و PO-146 و PO-255 و PO-0707 مدفوعة) لم تُحتسب كدعم لأنها سُددت.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="A19:E19"/>
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A14:E14"/>
     <mergeCell ref="A9:E9"/>
-    <mergeCell ref="A17:E17"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1089,13 +1084,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
     <col width="70" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -1109,32 +1104,32 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>أولاً: المسحوبات المباشرة من مزرعة الرياض (مديونية على نسما/أبو مازن)</t>
+          <t>أولاً: المسحوبات المباشرة (مديونية على أبو مازن)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="25" t="inlineStr">
         <is>
           <t>م</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="25" t="inlineStr">
         <is>
           <t>البند</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="25" t="inlineStr">
         <is>
           <t>المبلغ</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="D4" s="25" t="inlineStr">
         <is>
           <t>المصدر</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
+      <c r="E4" s="25" t="inlineStr">
         <is>
           <t>ملاحظة</t>
         </is>
@@ -1146,7 +1141,7 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>ترحيلات من الرياض إلى تبوك RNT (30-7-2025 إلى 31-7-2026)</t>
+          <t>ترحيلات من الرياض إلى تبوك RNT</t>
         </is>
       </c>
       <c r="C5" s="13" t="n">
@@ -1159,7 +1154,7 @@
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>⚠ بقيم النظام (القديم شامل ضريبة/الجديد بدون). شيت المحاسب بأسعار التحويل: 334,662.95 لـ RNT+RNP مع سندات ناقصة</t>
+          <t>⚠ بقيم النظام – شيت المحاسب بأسعار التحويل مختلف</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1164,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>ترحيلات إلى قسم المشاريع تبوك RNP (30-7-2025 إلى 31-7-2026)</t>
+          <t>ترحيلات إلى قسم المشاريع تبوك RNP</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
@@ -1180,11 +1175,7 @@
           <t>ملف حركات المواد – بقيم النظام</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>يشمل 17 سند ISV أُضيفت من ملف التفصيل</t>
-        </is>
-      </c>
+      <c r="E6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
@@ -1200,7 +1191,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>ملف مراجعة المسحوبات – شيت المصاريف الإدارية</t>
+          <t>ملف مراجعة المسحوبات</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr"/>
@@ -1211,7 +1202,7 @@
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>مسحوبات قبل الفترة – أوامر شراء P00480 إلى P00523 (102,875 حبة)</t>
+          <t>مسحوبات قبل الفترة – أوامر P00480 إلى P00523 (102,875 حبة)</t>
         </is>
       </c>
       <c r="C8" s="13" t="n">
@@ -1219,7 +1210,7 @@
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>ملف مراجعة المسحوبات – مسحوبات قبل الفترة</t>
+          <t>ملف مراجعة المسحوبات</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr">
@@ -1245,32 +1236,32 @@
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>ثانياً: المبالغ التي دعمت بها نسما/أبو مازن مزرعة الرياض (حق لنسما)</t>
+          <t>ثانياً: المسحوبات النقدية (مديونية على أبو مازن)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="25" t="inlineStr">
         <is>
           <t>م</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="25" t="inlineStr">
         <is>
           <t>البند</t>
         </is>
       </c>
-      <c r="C12" s="11" t="inlineStr">
+      <c r="C12" s="25" t="inlineStr">
         <is>
           <t>المبلغ</t>
         </is>
       </c>
-      <c r="D12" s="11" t="inlineStr">
+      <c r="D12" s="25" t="inlineStr">
         <is>
           <t>المصدر</t>
         </is>
       </c>
-      <c r="E12" s="11" t="inlineStr">
+      <c r="E12" s="25" t="inlineStr">
         <is>
           <t>ملاحظة</t>
         </is>
@@ -1282,21 +1273,20 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>ترحيلات من تبوك إلى الرياض TNR (30-7-2025 إلى 31-7-2026)</t>
+          <t>إيداع في حساب أبو مازن من إيرادات المناديب قبل الفترة</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>91545.48</v>
+        <v>197452</v>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>ملف حركات المواد – بقيم النظام</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>شيت المحاسب: 32,450 فقط (ناقص TNR-2689 و TNR-2888 و TRF-0188)</t>
-        </is>
+          <t>بيان صاحب الحساب</t>
+        </is>
+      </c>
+      <c r="E13" s="3">
+        <f> إيرادات 610,688 − مصروفات تشغيل دفعها م/ عادل 413,236 ✓</f>
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -1305,15 +1295,15 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>مصروفات إدارية 2025 (إقامات وتأشيرات ونقل كفالات)</t>
+          <t>منصرف 100,000 بتعليمات أبو مازن (9-3-2026)</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>56125</v>
+        <v>100000</v>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>كشف المصاريف الإدارية – البنود 49–55</t>
+          <t>كشف الخزنة – مصروف 131</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr"/>
@@ -1324,174 +1314,212 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>مصروفات إدارية وحكومية 2026 حتى 31-7 (تشمل إيجار المزرعة 150,000)</t>
+          <t>توريد نقدي للإدارة – أبو مازن (21-5-2026)</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>173979.15</v>
+        <v>13000</v>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>تقرير العهدة – المصروفات الإدارية</t>
+          <t>كشف الخزنة – مصروف 157</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="B16" s="12" t="inlineStr">
-        <is>
-          <t>ديزل سيارتي المناديب (11-2025 إلى 7-2026)</t>
-        </is>
-      </c>
-      <c r="C16" s="13" t="n">
-        <v>35141.98</v>
-      </c>
-      <c r="D16" s="12" t="inlineStr">
-        <is>
-          <t>شيت الديزل المدفوع من نسما</t>
-        </is>
-      </c>
-      <c r="E16" s="12" t="inlineStr">
-        <is>
-          <t>⚠ قد يتداخل مع ديزل العهد النقدية</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="B17" s="12" t="inlineStr">
-        <is>
-          <t>مشتريات 2025 مدفوعة بتحويل بنكي من تبوك</t>
-        </is>
-      </c>
-      <c r="C17" s="13" t="n">
-        <v>226679.26</v>
-      </c>
-      <c r="D17" s="12" t="inlineStr">
-        <is>
-          <t>ملف مصروفات 2025 – فلتر تحويل بنكي</t>
-        </is>
-      </c>
-      <c r="E17" s="12" t="inlineStr">
-        <is>
-          <t>⚠ الرقم اليدوي بالملف 269,099.26 (فرق 42,420 بدون حركات)</t>
-        </is>
-      </c>
+      <c r="A16" s="14" t="inlineStr"/>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>الإجمالي</t>
+        </is>
+      </c>
+      <c r="C16" s="15">
+        <f>SUM(C13:C15)</f>
+        <v/>
+      </c>
+      <c r="D16" s="14" t="n"/>
+      <c r="E16" s="14" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>مصروفات تأسيس مدفوعة عن طريق أبومازن (البنود 1 و 2 و 14)</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="n">
-        <v>133770</v>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>ثالثاً: دعم أبو مازن / نسما لمزرعة الرياض (حق له)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="25" t="inlineStr">
+        <is>
+          <t>م</t>
+        </is>
+      </c>
+      <c r="B19" s="25" t="inlineStr">
+        <is>
+          <t>البند</t>
+        </is>
+      </c>
+      <c r="C19" s="25" t="inlineStr">
+        <is>
+          <t>المبلغ</t>
+        </is>
+      </c>
+      <c r="D19" s="25" t="inlineStr">
+        <is>
+          <t>المصدر</t>
+        </is>
+      </c>
+      <c r="E19" s="25" t="inlineStr">
+        <is>
+          <t>ملاحظة</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>مصروفات التأسيس كاملة</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="n">
+        <v>1089735.8</v>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
         <is>
           <t>كشف مصروفات التأسيس</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>البند 14 (35,000) لسليمان الخضيري بتوجيه أبومازن</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="14" t="inlineStr"/>
-      <c r="B19" s="14" t="inlineStr">
-        <is>
-          <t>الإجمالي</t>
-        </is>
-      </c>
-      <c r="C19" s="15">
-        <f>SUM(C13:C18)</f>
-        <v/>
-      </c>
-      <c r="D19" s="14" t="n"/>
-      <c r="E19" s="14" t="n"/>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>⚠ البند 23 (دينة عماد 123,000) تاريخه 1-11-2025</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>ثالثاً: مسحوبات نقدية من خزنة مزرعة الرياض (مديونية على نسما/أبو مازن)</t>
-        </is>
-      </c>
+      <c r="A21" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>ترحيلات من تبوك إلى الرياض TNR</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>91545.48</v>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>ملف حركات المواد – بقيم النظام</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="inlineStr">
-        <is>
-          <t>م</t>
-        </is>
-      </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>البند</t>
-        </is>
-      </c>
-      <c r="C22" s="11" t="inlineStr">
-        <is>
-          <t>المبلغ</t>
-        </is>
-      </c>
-      <c r="D22" s="11" t="inlineStr">
-        <is>
-          <t>المصدر</t>
-        </is>
-      </c>
-      <c r="E22" s="11" t="inlineStr">
-        <is>
-          <t>ملاحظة</t>
-        </is>
-      </c>
+      <c r="A22" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>مصروفات إدارية 2025</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>56125</v>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>كشف المصاريف الإدارية</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>توريد نقدي للإدارة – أبو مازن (21-5-2026)</t>
+          <t>مصروفات إدارية وحكومية 2026 (تشمل إيجار المزرعة 150,000)</t>
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>13000</v>
+        <v>173979.15</v>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>كشف الخزنة – مصروف رقم 157</t>
+          <t>تقرير العهدة الإدارية</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="14" t="inlineStr"/>
-      <c r="B24" s="14" t="inlineStr">
+      <c r="A24" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>ديزل مدفوع من نسما</t>
+        </is>
+      </c>
+      <c r="C24" s="13" t="n">
+        <v>35141.98</v>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>شيت الديزل</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="inlineStr">
+        <is>
+          <t>⚠ قد يتداخل مع ديزل العهد</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>مشتريات 2025 مدفوعة من نسما (تحويل بنكي)</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="n">
+        <v>226679.26</v>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>ملف مصروفات 2025</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>⚠ الرقم اليدوي بالملف 269,099.26 (فرق 42,420 بدون حركات)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr"/>
+      <c r="B26" s="14" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="C24" s="15">
-        <f>SUM(C23:C23)</f>
-        <v/>
-      </c>
-      <c r="D24" s="14" t="n"/>
-      <c r="E24" s="14" t="n"/>
+      <c r="C26" s="15">
+        <f>SUM(C20:C25)</f>
+        <v/>
+      </c>
+      <c r="D26" s="14" t="n"/>
+      <c r="E26" s="14" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A11:E11"/>
-    <mergeCell ref="A21:E21"/>
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A18:E18"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1504,120 +1532,155 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
     <col width="70" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>بنود دعم لمزرعة الرياض غير محدد من دفعها من الشريكين</t>
+          <t>إيرادات ومصروفات المزرعة قبل 30-7-2025 (ليست دعماً من أي شريك)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>مدفوعة من حسابات بنكية (البنك السعودي / بنك الرياض / بنك ساب) – لم يُذكر صاحب الحساب</t>
+          <t>التسوية</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="25" t="inlineStr">
         <is>
           <t>م</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="25" t="inlineStr">
         <is>
           <t>البند</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="25" t="inlineStr">
         <is>
           <t>المبلغ</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="D4" s="25" t="inlineStr">
         <is>
           <t>المصدر</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
+      <c r="E4" s="25" t="inlineStr">
         <is>
           <t>ملاحظة</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="n">
+      <c r="A5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>مصروفات التأسيس – البنود المدفوعة من البنوك</t>
-        </is>
-      </c>
-      <c r="C5" s="13" t="n">
-        <v>955965.8</v>
-      </c>
-      <c r="D5" s="12" t="inlineStr">
-        <is>
-          <t>كشف مصروفات التأسيس (1,089,735.80 − 133,770 أبومازن)</t>
-        </is>
-      </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>⚠ يلزم تحديد أصحاب الحسابات البنكية. البند 23 (دينة عماد 123,000) تاريخه 1-11-2025</t>
-        </is>
-      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>إيرادات المناديب (1-10-2024 إلى 30-6-2025)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>610688</v>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>ملف المبيعات</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="n">
+      <c r="A6" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>مصروفات تشغيل قبل الفترة (2-2024 إلى 12-2024)</t>
-        </is>
-      </c>
-      <c r="C6" s="13" t="n">
-        <v>412040.67</v>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>كشف مصروفات التشغيل قبل 30.7.2025</t>
-        </is>
-      </c>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>⚠ مدفوعة من البنك السعودي وبنك الرياض</t>
-        </is>
-      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>يُخصم: مصروفات تشغيل دفعها م/ عادل من الإيرادات</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>-413236</v>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>ملف المصاريف التشغيلية</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr"/>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="A7" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>يُخصم: المودع في حساب أبو مازن</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>-197452</v>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>بيان صاحب الحساب</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>مُدرج كمسحوبات نقدية على أبو مازن</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr"/>
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="C7" s="15">
-        <f>SUM(C5:C6)</f>
-        <v/>
-      </c>
-      <c r="D7" s="14" t="n"/>
-      <c r="E7" s="14" t="n"/>
+      <c r="C8" s="15">
+        <f>SUM(C5:C7)</f>
+        <v/>
+      </c>
+      <c r="D8" s="14" t="n"/>
+      <c r="E8" s="14" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>الصافي = صفر ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>مصروفات تشغيل 2-2024 إلى 12-2024 (412,040.67) صُرفت من إيرادات المزرعة – لا تُحتسب دعماً لأي شريك.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B11:E11"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>